<commit_message>
feat: del drugs and update store UI
</commit_message>
<xml_diff>
--- a/Assets/Config/GameBalance.xlsx
+++ b/Assets/Config/GameBalance.xlsx
@@ -728,17 +728,6 @@
         <x:v>30</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="4" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B25" s="4">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C25" s="4" t="s">
-        <x:v>32</x:v>
-      </x:c>
-    </x:row>
     <x:row r="26">
       <x:c r="A26" s="3" t="s">
         <x:v>33</x:v>
@@ -863,17 +852,6 @@
         <x:v>49</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="3" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="B8" s="3">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="s">
-        <x:v>51</x:v>
-      </x:c>
-    </x:row>
     <x:row r="11">
       <x:c r="A11" s="4" t="s">
         <x:v>52</x:v>

</xml_diff>